<commit_message>
Modification in src folder files
</commit_message>
<xml_diff>
--- a/docs/Apollo_Camera_Laser_Network_Configuration_Report_Updated.xlsx
+++ b/docs/Apollo_Camera_Laser_Network_Configuration_Report_Updated.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YerriswamyChakala\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YerriswamyChakala\Desktop\Apollo_Application\Apollo_patch_pos\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04126691-610D-45C6-8688-33D7505C95C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF56CA91-88DE-4AE4-A612-141EF4900EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="173">
   <si>
     <t>Apollo Camera &amp; Laser Network Configuration Summary</t>
   </si>
@@ -275,9 +275,6 @@
     <t>TRI02KA-M</t>
   </si>
   <si>
-    <t>250500042</t>
-  </si>
-  <si>
     <t>Port 10</t>
   </si>
   <si>
@@ -285,9 +282,6 @@
   </si>
   <si>
     <t>Sidewall 2 Camera</t>
-  </si>
-  <si>
-    <t>254901428</t>
   </si>
   <si>
     <t>VLAN 20</t>
@@ -606,7 +600,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -653,6 +647,18 @@
         <fgColor rgb="FFE2F0D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -666,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -691,14 +697,20 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -709,6 +721,9 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -716,7 +731,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <b/>
@@ -750,6 +765,9 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -768,7 +786,7 @@
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Device Role"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Model"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Serial Number"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Serial Number" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="VLAN"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Switch Port"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="PC NIC Adapter"/>
@@ -994,16 +1012,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="18">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -1024,16 +1042,16 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1290,16 +1308,16 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -1544,18 +1562,18 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -3929,24 +3947,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -4053,7 +4071,7 @@
       <c r="B4" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="10" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -4113,14 +4131,14 @@
       <c r="B5" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>83</v>
+      <c r="C5" s="10">
+        <v>254901428</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>70</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>72</v>
@@ -4129,7 +4147,7 @@
         <v>73</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>75</v>
@@ -4168,28 +4186,28 @@
     </row>
     <row r="6" spans="1:26" ht="28.5">
       <c r="A6" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="10">
+        <v>254901431</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>75</v>
@@ -4228,28 +4246,28 @@
     </row>
     <row r="7" spans="1:26" ht="28.5">
       <c r="A7" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="10">
         <v>254901430</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>90</v>
-      </c>
       <c r="G7" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>75</v>
@@ -6923,27 +6941,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18">
-      <c r="A1" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
+      <c r="A1" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="3" spans="1:9" ht="30">
       <c r="A3" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>59</v>
@@ -6966,13 +6984,13 @@
     </row>
     <row r="4" spans="1:9" ht="15">
       <c r="A4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C4" t="s">
         <v>123</v>
-      </c>
-      <c r="B4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C4" t="s">
-        <v>125</v>
       </c>
       <c r="D4" t="s">
         <v>75</v>
@@ -6984,24 +7002,24 @@
         <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>7</v>
       </c>
       <c r="I4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15">
       <c r="A5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C5" t="s">
         <v>127</v>
-      </c>
-      <c r="B5" t="s">
-        <v>174</v>
-      </c>
-      <c r="C5" t="s">
-        <v>129</v>
       </c>
       <c r="D5" t="s">
         <v>75</v>
@@ -7010,16 +7028,16 @@
         <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>7</v>
       </c>
       <c r="I5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15">
@@ -7027,10 +7045,10 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D6" t="s">
         <v>75</v>
@@ -7039,16 +7057,16 @@
         <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>133</v>
-      </c>
       <c r="I6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -7078,16 +7096,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
-      <c r="A1" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
+      <c r="A1" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -7137,7 +7155,7 @@
     </row>
     <row r="3" spans="1:26" ht="15">
       <c r="A3" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>55</v>
@@ -7146,7 +7164,7 @@
         <v>54</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>59</v>
@@ -7155,7 +7173,7 @@
         <v>60</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>3</v>
@@ -7180,29 +7198,29 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="28.5">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="G4" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="H4" s="11" t="s">
         <v>102</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -7224,29 +7242,29 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="28.5">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="12" t="s">
         <v>102</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
@@ -7269,28 +7287,28 @@
     </row>
     <row r="6" spans="1:26" ht="28.5">
       <c r="A6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>75</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -7340,16 +7358,16 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26">
-      <c r="A8" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
+      <c r="A8" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -7374,7 +7392,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -7406,7 +7424,7 @@
         <v>25</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -7438,7 +7456,7 @@
         <v>27</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -7470,7 +7488,7 @@
         <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -7502,7 +7520,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -7559,7 +7577,7 @@
     </row>
     <row r="15" spans="1:26" ht="15">
       <c r="A15" s="7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -7589,7 +7607,7 @@
     </row>
     <row r="16" spans="1:26" ht="30">
       <c r="A16" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>55</v>
@@ -7598,7 +7616,7 @@
         <v>54</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>59</v>
@@ -7633,16 +7651,16 @@
     </row>
     <row r="17" spans="1:26" ht="15">
       <c r="A17" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>70</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>75</v>
@@ -7654,7 +7672,7 @@
         <v>7</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -7677,16 +7695,16 @@
     </row>
     <row r="18" spans="1:26" ht="15">
       <c r="A18" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>75</v>
@@ -7698,7 +7716,7 @@
         <v>7</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
@@ -7724,13 +7742,13 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>75</v>
@@ -7739,10 +7757,10 @@
         <v>76</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -7793,7 +7811,7 @@
     </row>
     <row r="21" spans="1:26">
       <c r="A21" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -7823,26 +7841,26 @@
     </row>
     <row r="22" spans="1:26">
       <c r="A22" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>75</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -7865,26 +7883,26 @@
     </row>
     <row r="23" spans="1:26">
       <c r="A23" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>75</v>
       </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
@@ -10087,14 +10105,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="A1" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -10140,22 +10158,22 @@
     </row>
     <row r="3" spans="1:23" ht="15">
       <c r="A3" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>145</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>147</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -10177,7 +10195,7 @@
     </row>
     <row r="4" spans="1:23" ht="15">
       <c r="A4" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>67</v>
@@ -10186,10 +10204,10 @@
         <v>74</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F4" s="3">
         <v>46176.499265787039</v>
@@ -10214,19 +10232,19 @@
     </row>
     <row r="5" spans="1:23" ht="15">
       <c r="A5" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F5" s="3">
         <v>46176.499265787039</v>
@@ -10251,19 +10269,19 @@
     </row>
     <row r="6" spans="1:23" ht="15">
       <c r="A6" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="F6" s="3">
         <v>46176.499265787039</v>
@@ -10288,19 +10306,19 @@
     </row>
     <row r="7" spans="1:23" ht="15">
       <c r="A7" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>150</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="F7" s="3">
         <v>46176.499265787039</v>
@@ -10325,19 +10343,19 @@
     </row>
     <row r="8" spans="1:23" ht="15">
       <c r="A8" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>156</v>
       </c>
       <c r="F8" s="3">
         <v>46176.499265787039</v>
@@ -10362,19 +10380,19 @@
     </row>
     <row r="9" spans="1:23" ht="30">
       <c r="A9" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>159</v>
       </c>
       <c r="F9" s="3">
         <v>46176.499265787039</v>
@@ -10399,19 +10417,19 @@
     </row>
     <row r="10" spans="1:23" ht="15">
       <c r="A10" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="D10" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F10" s="3">
         <v>46181.503053599539</v>
@@ -10436,19 +10454,19 @@
     </row>
     <row r="11" spans="1:23" ht="15">
       <c r="A11" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>129</v>
-      </c>
       <c r="D11" s="5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F11" s="3">
         <v>46181.503053599539</v>
@@ -10473,19 +10491,19 @@
     </row>
     <row r="12" spans="1:23" ht="30">
       <c r="A12" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F12" s="3">
         <v>46181.503053599539</v>
@@ -10510,19 +10528,19 @@
     </row>
     <row r="13" spans="1:23" ht="28.5">
       <c r="A13" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="D13" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>167</v>
       </c>
       <c r="F13" s="3">
         <v>46181.503053599539</v>

</xml_diff>